<commit_message>
Fixed time table and title defense slides
</commit_message>
<xml_diff>
--- a/Slides/Project-II.xlsx
+++ b/Slides/Project-II.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project-II\Slides\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project-ii-main\Slides\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7FC84224-4C81-42B7-A47E-098FA050EACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4664311E-8522-42B5-B563-0E1298771727}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{64BA5A5C-A07F-4473-9C99-22FB2828A215}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{64BA5A5C-A07F-4473-9C99-22FB2828A215}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -71,18 +71,12 @@
     <t>Proposal Defense</t>
   </si>
   <si>
-    <t>DFD Diagram</t>
-  </si>
-  <si>
     <t>Preparation of Documentation and Presentation</t>
   </si>
   <si>
     <t>Mid-Term Defense</t>
   </si>
   <si>
-    <t>UML Diagrams and Backlog</t>
-  </si>
-  <si>
     <t>Gantt chart</t>
   </si>
   <si>
@@ -141,6 +135,12 @@
   </si>
   <si>
     <t>PROJECT SUBMISSION DEADLINE: 12 July</t>
+  </si>
+  <si>
+    <t>UML Diagrams</t>
+  </si>
+  <si>
+    <t>Backlog</t>
   </si>
 </sst>
 </file>
@@ -251,9 +251,6 @@
     <xf numFmtId="16" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -262,6 +259,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -707,7 +707,7 @@
         <v>2.1</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C7" s="6">
         <v>46142</v>
@@ -725,17 +725,17 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="C8" s="6">
         <v>46145</v>
       </c>
       <c r="D8" s="6">
-        <v>46147</v>
+        <v>46148</v>
       </c>
       <c r="E8" s="4">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
@@ -743,17 +743,17 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="C9" s="6">
-        <v>46148</v>
+        <v>46149</v>
       </c>
       <c r="D9" s="6">
         <v>46149</v>
       </c>
       <c r="E9" s="4">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -761,7 +761,7 @@
         <v>2.4</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C10" s="6">
         <v>46150</v>
@@ -779,7 +779,7 @@
         <v>3</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C11" s="6"/>
       <c r="D11" s="6"/>
@@ -790,7 +790,7 @@
         <v>3.1</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C12" s="6">
         <v>46156</v>
@@ -808,7 +808,7 @@
         <v>3.2</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C13" s="6">
         <v>46160</v>
@@ -820,28 +820,28 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="K13" s="11" t="s">
-        <v>33</v>
+      <c r="K13" s="10" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="9">
+      <c r="A14" s="8">
         <v>3.3</v>
       </c>
-      <c r="B14" s="8" t="s">
-        <v>16</v>
+      <c r="B14" s="7" t="s">
+        <v>14</v>
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="6"/>
       <c r="E14" s="4"/>
-      <c r="K14" s="7"/>
+      <c r="K14" s="11"/>
     </row>
     <row r="15" spans="1:11" ht="21" x14ac:dyDescent="0.4">
       <c r="A15" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C15" s="6">
         <v>46162</v>
@@ -853,14 +853,14 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="K15" s="10"/>
+      <c r="K15" s="9"/>
     </row>
     <row r="16" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C16" s="6">
         <v>46165</v>
@@ -875,10 +875,10 @@
     </row>
     <row r="17" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="5" t="s">
         <v>21</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>23</v>
       </c>
       <c r="C17" s="6">
         <v>46168</v>
@@ -893,10 +893,10 @@
     </row>
     <row r="18" spans="1:6" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C18" s="6">
         <v>46170</v>
@@ -909,7 +909,7 @@
         <v>2</v>
       </c>
       <c r="F18" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
@@ -917,7 +917,7 @@
         <v>3.4</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C19" s="6">
         <v>46172</v>
@@ -930,7 +930,7 @@
         <v>4</v>
       </c>
       <c r="F19" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
@@ -938,7 +938,7 @@
         <v>3.5</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C20" s="6">
         <v>46176</v>
@@ -951,7 +951,7 @@
         <v>2</v>
       </c>
       <c r="F20" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
@@ -959,7 +959,7 @@
         <v>3.6</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C21" s="6">
         <v>46178</v>
@@ -990,7 +990,7 @@
         <v>2</v>
       </c>
       <c r="F22" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">

</xml_diff>